<commit_message>
Cambio en el vector estado
</commit_message>
<xml_diff>
--- a/docs/Libro1.xlsx
+++ b/docs/Libro1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CV\biblioteca-utn\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39A3221F-8A63-470F-9D3B-2B69D4D4A0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A4B9B6-1D1D-478F-98B8-7B0A170A24FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9947CA60-4663-463B-92CB-B5511348D704}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Evento</t>
   </si>
@@ -122,13 +122,31 @@
   <si>
     <t>AC personas
 retiradas</t>
+  </si>
+  <si>
+    <t>fin_lectura</t>
+  </si>
+  <si>
+    <t>RND tiempo de lectura</t>
+  </si>
+  <si>
+    <t>Tiempo lectura</t>
+  </si>
+  <si>
+    <t>RND Post prestamo</t>
+  </si>
+  <si>
+    <t>Proxima fin lectura</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Post prestamo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,8 +154,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -180,6 +206,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -193,21 +225,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -216,9 +239,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,116 +589,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83036F86-413E-41BB-B929-00B2235ADE6E}">
-  <dimension ref="B1:X5"/>
+  <dimension ref="B1:AC5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.5703125" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.28515625" customWidth="1"/>
-    <col min="20" max="20" width="22.42578125" customWidth="1"/>
+    <col min="8" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" customWidth="1"/>
+    <col min="14" max="14" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.28515625" customWidth="1"/>
+    <col min="25" max="25" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="D1" s="4" t="s">
+    <row r="1" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="D1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="5" t="s">
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
     </row>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="D2" s="3" t="s">
+    <row r="2" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="D2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="1" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2" t="s">
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="7" t="s">
+      <c r="U2" s="1"/>
+      <c r="V2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="W2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="X2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="2"/>
-      <c r="U2" s="8" t="s">
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
     </row>
-    <row r="3" spans="2:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3">
+    <row r="3" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3">
         <v>1</v>
       </c>
-      <c r="M3">
+      <c r="R3">
         <v>2</v>
       </c>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2">
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="1">
         <v>1</v>
       </c>
-      <c r="V3" s="2"/>
-      <c r="W3">
+      <c r="AA3" s="1"/>
+      <c r="AB3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -682,54 +739,69 @@
         <v>3</v>
       </c>
       <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4" t="s">
         <v>21</v>
       </c>
-      <c r="I4" t="s">
+      <c r="N4" t="s">
         <v>25</v>
       </c>
-      <c r="J4">
+      <c r="O4">
         <v>1</v>
       </c>
-      <c r="K4">
+      <c r="P4">
         <v>2</v>
       </c>
-      <c r="L4" t="s">
+      <c r="Q4" t="s">
         <v>7</v>
       </c>
-      <c r="M4" t="s">
+      <c r="R4" t="s">
         <v>7</v>
       </c>
-      <c r="N4" t="s">
+      <c r="S4" t="s">
         <v>6</v>
       </c>
-      <c r="O4" t="s">
+      <c r="T4" t="s">
         <v>9</v>
-      </c>
-      <c r="P4" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="7"/>
-      <c r="S4" t="s">
-        <v>14</v>
-      </c>
-      <c r="T4" t="s">
-        <v>15</v>
       </c>
       <c r="U4" t="s">
         <v>7</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="1"/>
+      <c r="W4" s="4"/>
+      <c r="X4" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>7</v>
+      </c>
+      <c r="AA4" t="s">
         <v>23</v>
       </c>
-      <c r="W4" t="s">
+      <c r="AB4" t="s">
         <v>7</v>
       </c>
-      <c r="X4" t="s">
+      <c r="AC4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>12</v>
       </c>
@@ -739,21 +811,23 @@
       <c r="F5">
         <v>4</v>
       </c>
+      <c r="H5" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="S2:T3"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="O2:P3"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="D1:K1"/>
-    <mergeCell ref="H2:K3"/>
+  <mergeCells count="13">
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="T2:U3"/>
+    <mergeCell ref="Q1:U1"/>
+    <mergeCell ref="D1:P1"/>
+    <mergeCell ref="M2:P3"/>
     <mergeCell ref="D2:G3"/>
+    <mergeCell ref="H2:L3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="Z2:AC2"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="X2:Y3"/>
+    <mergeCell ref="W2:W4"/>
+    <mergeCell ref="V2:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>